<commit_message>
Update survey data, wrangling scripts, and consolidate formatted output files
</commit_message>
<xml_diff>
--- a/Analysis/clean data/Survey 2_scored_near complete_16.6.26.xlsx
+++ b/Analysis/clean data/Survey 2_scored_near complete_16.6.26.xlsx
@@ -520,7 +520,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Adrià López-Baucells</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -570,7 +570,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Adrià López-Baucells albaucells@mcng.cat</t>
+          <t>AB</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Alexandra Howard</t>
+          <t>AH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -710,7 +710,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Alexandra Howard, alex.asterhof@gmail.com</t>
+          <t>AH</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -780,7 +780,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Andrés Muñoz-Sáez</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Andrés Muñoz-Sáez, andrmunoz@uchile.cl</t>
+          <t>AS</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>April Reside</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -955,7 +955,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>April Reside a.reside@uq.edu.au</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Ara Monadjem</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Ara Monadjem ara.monadjem@up.ac.za</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Brooke Maslo</t>
+          <t>BM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Brooke Maslo, brooke.maslo@rutgers.edu</t>
+          <t>BM</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Carme Tuneu-Corral</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Carme Tuneu-Corral - email: tuneucorral@gmail.com</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Carme Tuneu-Corral</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1500,7 +1500,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Carme Tuneu-Corral - tuneucorral@gmail.com</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1570,7 +1570,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1830,7 +1830,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1965,7 +1965,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2105,7 +2105,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2360,7 +2360,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2495,7 +2495,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2630,7 +2630,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2680,7 +2680,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Carmi Korine</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Carmi Korine, ckorine@bgu.ac.il</t>
+          <t>CK</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cárol Sierra-Durán</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3082,7 +3082,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Cárol Sierra-Durán camsierradu@unal.edu.co</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cárol Sierra-Durán</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Cárol Sierra-Durán camsierradu@unal.edu.co</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -3292,7 +3292,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Carolina Ocampo-Ariza</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Carolina Ocampo carocampoa@gmail.com</t>
+          <t>CO</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cecilia Montauban</t>
+          <t>CM</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Cecilia Montauban - montauc50@gmail.com</t>
+          <t>CM</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Danilo Russo</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Danilo Russo; danrusso@unina.it</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3652,7 +3652,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Diogo Ferreira</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Diogo Ferreira; ferreiradfa@gmail.com</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3782,7 +3782,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kadambari Deshpande</t>
+          <t>KD</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Dr. Kadambari Deshpande, Email: kadambari.deshpande@iihs.ac.in</t>
+          <t>KD</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Elisa Fuentes-Montemayor</t>
+          <t>EF</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Elisa Fuentes-Montemayor &lt;elisa.fuentes-montemayor@stir.ac.uk&gt;</t>
+          <t>EF</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Florence Matutini</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4107,8 +4107,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Florence Matutini
- florence.matutini@ofb.gouv.fr</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -4173,7 +4172,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Florence Matutini</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4223,8 +4222,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Florence Matutini
- florence.matutini@ofb.gouv.fr</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4294,7 +4292,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Florence Matutini</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4344,8 +4342,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Florence Matutini
- florence.matutini@ofb.gouv.fr</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -4410,7 +4407,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gary McCracken</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -4460,7 +4457,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Gary McCracken</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -4545,7 +4542,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gary McCracken</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -4595,7 +4592,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Gary McCracken</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -4675,7 +4672,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Heidi Kolkert</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -4725,7 +4722,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Heidi Kolkert, hkolker2@une.edu.au</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4815,7 +4812,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Heidi Kolkert</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4865,7 +4862,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Heidi Kolkert, hkolker2@une.edu.au</t>
+          <t>HK</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4960,7 +4957,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Hugo Rebelo</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5010,7 +5007,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Hugo Rebelo herebelo@fc.ul.pt</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -5095,7 +5092,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Hugo Rebelo</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5145,7 +5142,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Hugo Rebelo herebelo@fc.ul.pt</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -5215,7 +5212,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Hui Wu</t>
+          <t>HW</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5265,7 +5262,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Hui Wu wuh123@nenu.edu.cn</t>
+          <t>HW</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -5335,7 +5332,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jarod McTaggart</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5385,7 +5382,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Jarod jarodmctaggart1312@gmail.com @jaja1312</t>
+          <t>JM</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -5470,7 +5467,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jeremy Froidevaux</t>
+          <t>JF</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -5520,7 +5517,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Jeremy Froidevaux : jeremy.froidevaux@univ-fcomte.fr</t>
+          <t>JF</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -5601,7 +5598,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jérémy Froidevaux</t>
+          <t>JF</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -5651,7 +5648,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Jérémy Froidevaux : jeremy.froidevaux@univ-fcomte.fr</t>
+          <t>JF</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -5749,7 +5746,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Jian-Nan Liu</t>
+          <t>JN</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -5799,7 +5796,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Jian-Nan Liu</t>
+          <t>JN</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -5869,7 +5866,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>José M. Herrera</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -5919,7 +5916,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>José M. Herrera josemanuel.herrera@uca.es</t>
+          <t>JH</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -5989,7 +5986,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Leonardo Ancillotto</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6039,7 +6036,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Leonardo Ancillotto leonardo.ancillotto@cnr.it</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -6109,7 +6106,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Leonardo Ancillotto</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6159,7 +6156,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Leonardo Ancillotto leonardo.ancillotto@cnr.it</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -6229,7 +6226,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Maggie Campbell-Jones</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -6279,7 +6276,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Maggie Campbell-Jones mcampbelljones@usc.edu.au</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -6369,7 +6366,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Nayelli Rivera</t>
+          <t>N</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -6419,7 +6416,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Nayelli Rivera, a.riveravillanueva@student.uq.edu.au</t>
+          <t>N</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -6515,7 +6512,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Peter Taylor</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -6565,7 +6562,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Peter Taylor taylorpj@ufs.ac.za</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -6630,7 +6627,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Peter Taylor</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -6680,7 +6677,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Peter Taylor taylorpj@ufs.ac.za</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -6760,7 +6757,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Rani Davis</t>
+          <t>RD</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -6810,7 +6807,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Rani rani.davis@uq.net.au</t>
+          <t>RD</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -6905,7 +6902,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Sándor Zsebők</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -6955,7 +6952,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Sándor Zsebők zsebok.s@gmail.com</t>
+          <t>SZ</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -7025,7 +7022,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Siteri Tikoca</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -7075,7 +7072,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Siteri Tikoca- stikoca@gmail.com</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -7170,7 +7167,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Stuart Parsons</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -7220,7 +7217,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Stuart Parsons (stuart.parsons@canterbury.ac.nz)</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -7315,7 +7312,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Teja Tscharntke</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -7365,7 +7362,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Teja Tscharntke, ttschar@gwdg.de</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -7445,7 +7442,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Teja Tscharntke</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -7495,7 +7492,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Teja Tscharntke, ttschar@gwdg.de</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -7560,7 +7557,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Teja Tscharntke</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -7610,7 +7607,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Teja Tscharntke, ttschar@gwdg.de</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -7680,7 +7677,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Tinglei Jiang</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -7730,7 +7727,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Tinglei Jiang</t>
+          <t>TJ</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -7795,7 +7792,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Xavier Puig-Montserrat</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -7845,8 +7842,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Xavier Puig-Montserrat
-xavier.puig@uvic.cat</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -7931,7 +7927,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Xavier Puig-Montserrat</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -7981,8 +7977,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Xavier Puig-Montserrat
-xavier.puig@uvic.cat</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -8067,7 +8062,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Xavier Puig-Montserrat</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -8117,8 +8112,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Xavier Puig-Montserrat
-xavier.puig@uvic.cat</t>
+          <t>XP</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -8203,7 +8197,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Zenon Czenze &amp; Heidi Kolkert</t>
+          <t>ZC &amp; HK</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -8253,7 +8247,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Zenon Czenze, zczenze@une.edu.au; Heidi Kolkert &lt;hkolker2@une.edu.au&gt;</t>
+          <t>ZC &amp; HK</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -8343,7 +8337,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Helen Taylor-Boyd</t>
+          <t>HT</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -8353,7 +8347,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Helen Taylor-Boyd; batsinzambia@gmail.com</t>
+          <t>HT</t>
         </is>
       </c>
     </row>
@@ -8365,7 +8359,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Yingying Liu</t>
+          <t>YL</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -8375,7 +8369,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Yingying Liu; liuyy777@nenu.edu.cn</t>
+          <t>YL</t>
         </is>
       </c>
       <c r="V63" t="inlineStr">
@@ -8403,7 +8397,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Bea Maas</t>
+          <t>BM</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -8413,7 +8407,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Bea Maas bea.maas@univie.ac.at</t>
+          <t>BM</t>
         </is>
       </c>
     </row>
@@ -8425,7 +8419,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Olga Heim</t>
+          <t>OH</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -8435,7 +8429,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Olga Heim bats@o-heim.de &lt;bats@o-heim.de&gt;</t>
+          <t>OH</t>
         </is>
       </c>
     </row>
@@ -8447,7 +8441,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Kirsten Reichel-Jung</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -8457,7 +8451,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Dr Kirsten Reichel-Jung kirsten.jung@uni-ulm.de</t>
+          <t>KR</t>
         </is>
       </c>
     </row>
@@ -8469,7 +8463,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Chiara Paniccia</t>
+          <t>CP</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -8479,7 +8473,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Chiara Paniccia &lt;chiara.paniccia@eurac.edu&gt;</t>
+          <t>CP</t>
         </is>
       </c>
     </row>

</xml_diff>